<commit_message>
update smtpage and shanaz357
</commit_message>
<xml_diff>
--- a/sampledata/RLLT-Tabledata.xlsx
+++ b/sampledata/RLLT-Tabledata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\RLLT\Project-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\RLLT\Webapp\sampledata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390B5DAD-CE03-4801-96D0-4A8C78D0203B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B877CC5C-D147-487C-9CB3-D35A9F5C25E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5496" yWindow="5772" windowWidth="17280" windowHeight="5784" xr2:uid="{1B3B65C1-F353-4DCA-9F8A-394DBF5E61C5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1B3B65C1-F353-4DCA-9F8A-394DBF5E61C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,21 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t>1min</t>
   </si>
@@ -147,12 +138,100 @@
   <si>
     <t>Scheduled Days</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>O.T BKS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>N.T BKS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>WE5</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PRO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PSA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>CHP</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>VER</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7.5"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PPL</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,6 +261,12 @@
       <b/>
       <sz val="6.5"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="6.5"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -219,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -229,6 +314,18 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -545,13 +642,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBDA8A1D-2F67-48F6-8282-BC03DFE5A71D}">
-  <dimension ref="B2:G47"/>
+  <dimension ref="B2:T47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>26</v>
       </c>
@@ -570,8 +667,32 @@
       <c r="G2" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B3" s="1">
         <v>1</v>
       </c>
@@ -590,8 +711,21 @@
       <c r="G3" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="5"/>
+      <c r="T3" s="5"/>
+    </row>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B4" s="1">
         <v>1</v>
       </c>
@@ -610,8 +744,16 @@
       <c r="G4" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <v>1</v>
       </c>
@@ -630,8 +772,16 @@
       <c r="G5" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B6" s="1">
         <v>1</v>
       </c>
@@ -650,8 +800,16 @@
       <c r="G6" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <v>1</v>
       </c>
@@ -670,8 +828,16 @@
       <c r="G7" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B8" s="1">
         <v>1</v>
       </c>
@@ -690,8 +856,16 @@
       <c r="G8" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <v>1</v>
       </c>
@@ -710,8 +884,16 @@
       <c r="G9" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B10" s="1">
         <v>1</v>
       </c>
@@ -730,8 +912,16 @@
       <c r="G10" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B11" s="1">
         <v>1</v>
       </c>
@@ -750,8 +940,16 @@
       <c r="G11" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B12" s="1">
         <v>1</v>
       </c>
@@ -770,8 +968,16 @@
       <c r="G12" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <v>2</v>
       </c>
@@ -790,8 +996,16 @@
       <c r="G13" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B14" s="1">
         <v>2</v>
       </c>
@@ -810,8 +1024,16 @@
       <c r="G14" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B15" s="1">
         <v>2</v>
       </c>
@@ -830,8 +1052,16 @@
       <c r="G15" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B16" s="1">
         <v>2</v>
       </c>
@@ -850,8 +1080,16 @@
       <c r="G16" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="1">
         <v>2</v>
       </c>
@@ -870,8 +1108,16 @@
       <c r="G17" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="1">
         <v>2</v>
       </c>
@@ -890,8 +1136,16 @@
       <c r="G18" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="1">
         <v>2</v>
       </c>
@@ -910,8 +1164,16 @@
       <c r="G19" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="1">
         <v>2</v>
       </c>
@@ -930,8 +1192,16 @@
       <c r="G20" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="1">
         <v>2</v>
       </c>
@@ -950,8 +1220,16 @@
       <c r="G21" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="1">
         <v>2</v>
       </c>
@@ -970,8 +1248,16 @@
       <c r="G22" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="1">
         <v>2</v>
       </c>
@@ -990,8 +1276,16 @@
       <c r="G23" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+    </row>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B24" s="1">
         <v>2</v>
       </c>
@@ -1010,8 +1304,16 @@
       <c r="G24" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B25" s="1">
         <v>3</v>
       </c>
@@ -1030,8 +1332,16 @@
       <c r="G25" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="1">
         <v>3</v>
       </c>
@@ -1050,8 +1360,16 @@
       <c r="G26" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+    </row>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B27" s="1">
         <v>3</v>
       </c>
@@ -1070,8 +1388,16 @@
       <c r="G27" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+    </row>
+    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B28" s="1">
         <v>3</v>
       </c>
@@ -1090,8 +1416,16 @@
       <c r="G28" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B29" s="1">
         <v>3</v>
       </c>
@@ -1110,8 +1444,16 @@
       <c r="G29" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B30" s="1">
         <v>3</v>
       </c>
@@ -1130,8 +1472,16 @@
       <c r="G30" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B31" s="1">
         <v>3</v>
       </c>
@@ -1150,8 +1500,16 @@
       <c r="G31" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+    </row>
+    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B32" s="1">
         <v>3</v>
       </c>
@@ -1170,8 +1528,16 @@
       <c r="G32" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+    </row>
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B33" s="1">
         <v>3</v>
       </c>
@@ -1190,8 +1556,16 @@
       <c r="G33" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+    </row>
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B34" s="1">
         <v>3</v>
       </c>
@@ -1210,8 +1584,16 @@
       <c r="G34" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+    </row>
+    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B35" s="1">
         <v>3</v>
       </c>
@@ -1230,8 +1612,16 @@
       <c r="G35" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+    </row>
+    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B36" s="1">
         <v>4</v>
       </c>
@@ -1250,8 +1640,16 @@
       <c r="G36" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1"/>
+    </row>
+    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B37" s="1">
         <v>4</v>
       </c>
@@ -1270,8 +1668,16 @@
       <c r="G37" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B38" s="1">
         <v>4</v>
       </c>
@@ -1290,8 +1696,16 @@
       <c r="G38" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1"/>
+    </row>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B39" s="1">
         <v>4</v>
       </c>
@@ -1310,8 +1724,16 @@
       <c r="G39" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+    </row>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B40" s="1">
         <v>4</v>
       </c>
@@ -1330,8 +1752,16 @@
       <c r="G40" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
+      <c r="N40" s="1"/>
+      <c r="O40" s="1"/>
+    </row>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B41" s="1">
         <v>4</v>
       </c>
@@ -1350,8 +1780,16 @@
       <c r="G41" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="J41" s="1"/>
+      <c r="K41" s="1"/>
+      <c r="L41" s="1"/>
+      <c r="M41" s="1"/>
+      <c r="N41" s="1"/>
+      <c r="O41" s="1"/>
+    </row>
+    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B42" s="1">
         <v>4</v>
       </c>
@@ -1370,8 +1808,16 @@
       <c r="G42" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+      <c r="J42" s="1"/>
+      <c r="K42" s="1"/>
+      <c r="L42" s="1"/>
+      <c r="M42" s="1"/>
+      <c r="N42" s="1"/>
+      <c r="O42" s="1"/>
+    </row>
+    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B43" s="1">
         <v>5</v>
       </c>
@@ -1390,8 +1836,16 @@
       <c r="G43" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H43" s="1"/>
+      <c r="I43" s="1"/>
+      <c r="J43" s="1"/>
+      <c r="K43" s="1"/>
+      <c r="L43" s="1"/>
+      <c r="M43" s="1"/>
+      <c r="N43" s="1"/>
+      <c r="O43" s="1"/>
+    </row>
+    <row r="44" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B44" s="1">
         <v>5</v>
       </c>
@@ -1410,8 +1864,16 @@
       <c r="G44" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+      <c r="J44" s="1"/>
+      <c r="K44" s="1"/>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+      <c r="O44" s="1"/>
+    </row>
+    <row r="45" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B45" s="1">
         <v>5</v>
       </c>
@@ -1430,8 +1892,16 @@
       <c r="G45" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
+      <c r="J45" s="1"/>
+      <c r="K45" s="1"/>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1"/>
+      <c r="O45" s="1"/>
+    </row>
+    <row r="46" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B46" s="1">
         <v>5</v>
       </c>
@@ -1450,8 +1920,16 @@
       <c r="G46" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+      <c r="J46" s="1"/>
+      <c r="K46" s="1"/>
+      <c r="L46" s="1"/>
+      <c r="M46" s="1"/>
+      <c r="N46" s="1"/>
+      <c r="O46" s="1"/>
+    </row>
+    <row r="47" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B47" s="1">
         <v>5</v>
       </c>
@@ -1470,6 +1948,14 @@
       <c r="G47" s="2">
         <v>40</v>
       </c>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1"/>
+      <c r="J47" s="1"/>
+      <c r="K47" s="1"/>
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1"/>
+      <c r="O47" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>